<commit_message>
upd new extrx dataset
</commit_message>
<xml_diff>
--- a/logs/scaleup/summary/gpt-oss_simplyrx_ce_std_analysis.xlsx
+++ b/logs/scaleup/summary/gpt-oss_simplyrx_ce_std_analysis.xlsx
@@ -58,7 +58,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -430,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -443,18 +445,23 @@
           <t>gpt-oss simplyrx: CE vs STD</t>
         </is>
       </c>
+      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Analysis Dir</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>logs/scaleup/icl_gen_simplyrx/model=gpt-oss</t>
         </is>
       </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -501,74 +508,62 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>agentic_reflection coverage</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Current logs cover 89 runs, so some denominators are smaller than 105</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Overall Observations</t>
+        </is>
+      </c>
       <c r="B9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Overall Observations</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>CE / agentic_reflection is currently strongest at 0.819 = 86/105.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CE / agentic_reflection has the highest current solve rate: 0.831 = 74/89, but on only 89 available runs.</t>
+          <t>CE / single_inference is back to full coverage at 69/105 with solve rate 0.657; STD is 43/105 with solve rate 0.410.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Among methods with full 105-run coverage, CE / single_inference is strongest at 0.657 = 69/105; STD is weakest at 0.410 = 43/105.</t>
+          <t>Fully solved states x stardepth cells: agentic_reflection 27/35, single_inference 20/35, STD 12/35.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Fully solved states x stardepth cells: agentic_reflection 22/35, single_inference 20/35, STD 12/35.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>All methods are stable at StarDepth=0; performance drops as complexity rises, with agentic_reflection holding up best on more mid/high-difficulty cells.</t>
+          <t>All methods remain most stable at StarDepth=0; performance drops with complexity, while agentic_reflection holds up best on more mid/high-difficulty cells.</t>
         </is>
       </c>
     </row>
@@ -906,17 +901,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=23; r=4</t>
+          <t>3/3 [##########]; s=28; r=5</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=119; r=3</t>
+          <t>3/3 [##########]; s=112; r=4</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=61; r=7</t>
+          <t>3/3 [##########]; s=42; r=9</t>
         </is>
       </c>
     </row>
@@ -931,7 +926,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=32; r=6</t>
+          <t>3/3 [##########]; s=26; r=5</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -941,12 +936,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2/3 [#######---]; s=205.5; r=4</t>
+          <t>3/3 [##########]; s=245; r=4</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>1/2 [#####-----]; s=82; r=5</t>
+          <t>0/3 [----------]; s=NA; r=NA</t>
         </is>
       </c>
     </row>
@@ -961,22 +956,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=13; r=3</t>
+          <t>3/3 [##########]; s=14; r=3</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>1/2 [#####-----]; s=86; r=4</t>
+          <t>3/3 [##########]; s=54; r=3</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=25; r=5</t>
+          <t>3/3 [##########]; s=36; r=4</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=16; r=4</t>
+          <t>3/3 [##########]; s=12; r=3</t>
         </is>
       </c>
     </row>
@@ -991,22 +986,22 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=14; r=3</t>
+          <t>3/3 [##########]; s=16; r=5</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=16; r=3</t>
+          <t>3/3 [##########]; s=30; r=4</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=16; r=3</t>
+          <t>3/3 [##########]; s=25; r=5</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>0/1 [----------]; s=NA; r=NA</t>
+          <t>2/3 [#######---]; s=65.5; r=7</t>
         </is>
       </c>
     </row>
@@ -1021,22 +1016,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=21; r=7</t>
+          <t>3/3 [##########]; s=21; r=5</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>0/1 [----------]; s=NA; r=NA</t>
+          <t>0/3 [----------]; s=NA; r=NA</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>1/3 [###-------]; s=360; r=7</t>
+          <t>1/3 [###-------]; s=169; r=5</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>0/1 [----------]; s=NA; r=NA</t>
+          <t>1/3 [###-------]; s=378; r=8</t>
         </is>
       </c>
     </row>
@@ -1046,27 +1041,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>3/3 [##########]; s=12; r=2</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>3/3 [##########]; s=189; r=6</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>3/3 [##########]; s=520; r=9</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
           <t>3/3 [##########]; s=17; r=3</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>3/3 [##########]; s=92; r=5</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>0/1 [----------]; s=NA; r=NA</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>2/3 [#######---]; s=36.5; r=3.5</t>
-        </is>
-      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>0/1 [----------]; s=NA; r=NA</t>
+          <t>1/3 [###-------]; s=609; r=10</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1071,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=32; r=3</t>
+          <t>3/3 [##########]; s=18; r=3</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1086,17 +1081,17 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>1/2 [#####-----]; s=47; r=8</t>
+          <t>3/3 [##########]; s=27; r=4</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>0/2 [----------]; s=NA; r=NA</t>
+          <t>0/3 [----------]; s=NA; r=NA</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>0/1 [----------]; s=NA; r=NA</t>
+          <t>0/3 [----------]; s=NA; r=NA</t>
         </is>
       </c>
     </row>

</xml_diff>